<commit_message>
docs: explain C1 sell tracking triggers and parameters
</commit_message>
<xml_diff>
--- a/docs-C1-Sell/开发清单/looply-C1-Sell-埋点开发清单-v1.2.xlsx
+++ b/docs-C1-Sell/开发清单/looply-C1-Sell-埋点开发清单-v1.2.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf273073187e84881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详细点位" sheetId="2" r:id="Rccddbf06563643fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交互字典" sheetId="3" r:id="Rb0d2e5596fa04800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段复用" sheetId="4" r:id="R45c5b5540de2455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GA4映射" sheetId="5" r:id="R8a2f9db55e564cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举与验收" sheetId="6" r:id="Rb9d046608fb644ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1 UI对照" sheetId="7" r:id="Re882a1a8958a46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1a96d977a1e74af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详细点位" sheetId="2" r:id="R4438766da5c04d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交互字典" sheetId="3" r:id="R85d702b60cb84e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共字段复用" sheetId="4" r:id="Rffeef4b167f647cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GA4映射" sheetId="5" r:id="Ra3903b24acec4070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举与验收" sheetId="6" r:id="Rdae33656ccff40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1 UI对照" sheetId="7" r:id="Rf06dc5be9ba54a8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -564,6 +564,9 @@
       <x:c r="P3" s="20" t="str">
         <x:v>variant_id</x:v>
       </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>业务解释（触发时机 / 参数意义）</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -600,6 +603,9 @@
       <x:c r="N4" s="17" t="str"/>
       <x:c r="O4" s="17" t="str"/>
       <x:c r="P4" s="17" t="str"/>
+      <x:c r="Q4" t="str">
+        <x:v>页面实例真正到达并可见时记录；预加载、后台预取和同一页面实例重复渲染不算新的到达。参数用于标识页面（page_id）、页面实例（page_instance_id）和后续来源/设备分析。</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -650,6 +656,9 @@
       <x:c r="P5" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -700,6 +709,9 @@
       <x:c r="P6" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -747,6 +759,9 @@
       </x:c>
       <x:c r="P7" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -784,6 +799,9 @@
       <x:c r="N8" s="17" t="str"/>
       <x:c r="O8" s="17" t="str"/>
       <x:c r="P8" s="17" t="str"/>
+      <x:c r="Q8" t="str">
+        <x:v>内容进入前台并连续可见约 1 秒时记录一次；快速划过、预加载和同一页面实例同一内容重复出现不记录。参数用于说明内容模块、内容标识、位置及 ready/empty 状态。</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -832,6 +850,9 @@
       <x:c r="P9" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -879,6 +900,9 @@
       </x:c>
       <x:c r="P10" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -916,6 +940,9 @@
       <x:c r="N11" s="17" t="str"/>
       <x:c r="O11" s="17" t="str"/>
       <x:c r="P11" s="17" t="str"/>
+      <x:c r="Q11" t="str">
+        <x:v>内容进入前台并连续可见约 1 秒时记录一次；快速划过、预加载和同一页面实例同一内容重复出现不记录。参数用于说明内容模块、内容标识、位置及 ready/empty 状态。</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -966,6 +993,9 @@
       <x:c r="P12" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -1016,6 +1046,9 @@
       <x:c r="P13" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q13" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -1066,6 +1099,9 @@
       <x:c r="P14" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q14" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -1116,6 +1152,9 @@
       <x:c r="P15" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
@@ -1166,6 +1205,9 @@
       <x:c r="P16" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="36" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
@@ -1215,6 +1257,9 @@
       </x:c>
       <x:c r="P17" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q17" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1252,6 +1297,9 @@
       <x:c r="N18" s="17" t="str"/>
       <x:c r="O18" s="17" t="str"/>
       <x:c r="P18" s="17" t="str"/>
+      <x:c r="Q18" t="str">
+        <x:v>预约表单首次真正展示时记录；重新渲染、返回或刷新不重复记为开始。参数用于说明用户从哪里进入（entry_source）以及 ZIP/售卖方式是否已预填。</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
@@ -1288,6 +1336,9 @@
       <x:c r="N19" s="17" t="str"/>
       <x:c r="O19" s="17" t="str"/>
       <x:c r="P19" s="17" t="str"/>
+      <x:c r="Q19" t="str">
+        <x:v>预约流程某一步首次实际展示时记录；重渲染不重复，返回后再次真实到达按流程规则记录。flow_step 表示 Step 1–4，seller_flow_id 负责把步骤串成同一次预约流程。</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
@@ -1324,6 +1375,9 @@
       <x:c r="N20" s="17" t="str"/>
       <x:c r="O20" s="17" t="str"/>
       <x:c r="P20" s="17" t="str"/>
+      <x:c r="Q20" t="str">
+        <x:v>预约流程某一步首次实际展示时记录；重渲染不重复，返回后再次真实到达按流程规则记录。flow_step 表示 Step 1–4，seller_flow_id 负责把步骤串成同一次预约流程。</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
@@ -1360,6 +1414,9 @@
       <x:c r="N21" s="17" t="str"/>
       <x:c r="O21" s="17" t="str"/>
       <x:c r="P21" s="17" t="str"/>
+      <x:c r="Q21" t="str">
+        <x:v>预约流程某一步首次实际展示时记录；重渲染不重复，返回后再次真实到达按流程规则记录。flow_step 表示 Step 1–4，seller_flow_id 负责把步骤串成同一次预约流程。</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
@@ -1396,6 +1453,9 @@
       <x:c r="N22" s="17" t="str"/>
       <x:c r="O22" s="17" t="str"/>
       <x:c r="P22" s="17" t="str"/>
+      <x:c r="Q22" t="str">
+        <x:v>预约流程某一步首次实际展示时记录；重渲染不重复，返回后再次真实到达按流程规则记录。flow_step 表示 Step 1–4，seller_flow_id 负责把步骤串成同一次预约流程。</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
@@ -1446,6 +1506,9 @@
       <x:c r="P23" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q23" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
@@ -1496,6 +1559,9 @@
       <x:c r="P24" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q24" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
@@ -1545,6 +1611,9 @@
       </x:c>
       <x:c r="P25" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q25" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -1582,6 +1651,9 @@
       <x:c r="N26" s="17" t="str"/>
       <x:c r="O26" s="17" t="str"/>
       <x:c r="P26" s="17" t="str"/>
+      <x:c r="Q26" t="str">
+        <x:v>内容加载、草稿保存或恢复出现明确成功/失败终态时记录；Loading 中间态不记录。operation 说明发生了哪类操作，result_state/content_state 说明结果，失败时用 c1_failure_code 说明失败原因。</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
@@ -1618,6 +1690,9 @@
       <x:c r="N27" s="17" t="str"/>
       <x:c r="O27" s="17" t="str"/>
       <x:c r="P27" s="17" t="str"/>
+      <x:c r="Q27" t="str">
+        <x:v>内容加载、草稿保存或恢复出现明确成功/失败终态时记录；Loading 中间态不记录。operation 说明发生了哪类操作，result_state/content_state 说明结果，失败时用 c1_failure_code 说明失败原因。</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
@@ -1668,6 +1743,9 @@
       <x:c r="P28" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q28" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
@@ -1718,6 +1796,9 @@
       <x:c r="P29" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q29" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -1768,6 +1849,9 @@
       <x:c r="P30" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q30" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
@@ -1818,6 +1902,9 @@
       <x:c r="P31" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q31" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="24" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
@@ -1868,6 +1955,9 @@
       <x:c r="P32" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q32" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
@@ -1918,6 +2008,9 @@
       <x:c r="P33" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q33" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="36" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
@@ -1968,6 +2061,9 @@
       <x:c r="P34" s="17" t="str">
         <x:v>suggestion</x:v>
       </x:c>
+      <x:c r="Q34" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
@@ -2018,6 +2114,9 @@
       <x:c r="P35" s="17" t="str">
         <x:v>manual</x:v>
       </x:c>
+      <x:c r="Q35" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
@@ -2068,6 +2167,9 @@
       <x:c r="P36" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q36" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -2118,6 +2220,9 @@
       <x:c r="P37" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q37" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="24" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
@@ -2168,6 +2273,9 @@
       <x:c r="P38" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q38" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="24" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
@@ -2218,6 +2326,9 @@
       <x:c r="P39" s="17" t="str">
         <x:v>standalone</x:v>
       </x:c>
+      <x:c r="Q39" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="24" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
@@ -2268,6 +2379,9 @@
       <x:c r="P40" s="17" t="str">
         <x:v>step3</x:v>
       </x:c>
+      <x:c r="Q40" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="24" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
@@ -2317,6 +2431,9 @@
       </x:c>
       <x:c r="P41" s="17" t="str">
         <x:v>step4</x:v>
+      </x:c>
+      <x:c r="Q41" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
@@ -2354,6 +2471,9 @@
       <x:c r="N42" s="17" t="str"/>
       <x:c r="O42" s="17" t="str"/>
       <x:c r="P42" s="17" t="str"/>
+      <x:c r="Q42" t="str">
+        <x:v>ZIP 查询收到明确终态时记录；发起和 Loading 不算结果，自动网络重试沿用同一查询 ID，用户主动 Retry 才新建一次查询。query_context 说明查询发生在哪个页面/步骤，result_state 和 coverage_status 说明请求结果及是否覆盖。</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
@@ -2390,6 +2510,9 @@
       <x:c r="N43" s="17" t="str"/>
       <x:c r="O43" s="17" t="str"/>
       <x:c r="P43" s="17" t="str"/>
+      <x:c r="Q43" t="str">
+        <x:v>ZIP 查询收到明确终态时记录；发起和 Loading 不算结果，自动网络重试沿用同一查询 ID，用户主动 Retry 才新建一次查询。query_context 说明查询发生在哪个页面/步骤，result_state 和 coverage_status 说明请求结果及是否覆盖。</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -2426,6 +2549,9 @@
       <x:c r="N44" s="17" t="str"/>
       <x:c r="O44" s="17" t="str"/>
       <x:c r="P44" s="17" t="str"/>
+      <x:c r="Q44" t="str">
+        <x:v>ZIP 查询收到明确终态时记录；发起和 Loading 不算结果，自动网络重试沿用同一查询 ID，用户主动 Retry 才新建一次查询。query_context 说明查询发生在哪个页面/步骤，result_state 和 coverage_status 说明请求结果及是否覆盖。</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -2462,6 +2588,9 @@
       <x:c r="N45" s="17" t="str"/>
       <x:c r="O45" s="17" t="str"/>
       <x:c r="P45" s="17" t="str"/>
+      <x:c r="Q45" t="str">
+        <x:v>ZIP 查询收到明确终态时记录；发起和 Loading 不算结果，自动网络重试沿用同一查询 ID，用户主动 Retry 才新建一次查询。query_context 说明查询发生在哪个页面/步骤，result_state 和 coverage_status 说明请求结果及是否覆盖。</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
@@ -2512,6 +2641,9 @@
       <x:c r="P46" s="17" t="str">
         <x:v>standalone</x:v>
       </x:c>
+      <x:c r="Q46" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -2562,6 +2694,9 @@
       <x:c r="P47" s="17" t="str">
         <x:v>step3</x:v>
       </x:c>
+      <x:c r="Q47" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="24" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -2612,6 +2747,9 @@
       <x:c r="P48" s="17" t="str">
         <x:v>step4</x:v>
       </x:c>
+      <x:c r="Q48" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -2661,6 +2799,9 @@
       </x:c>
       <x:c r="P49" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q49" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -2698,6 +2839,9 @@
       <x:c r="N50" s="17" t="str"/>
       <x:c r="O50" s="17" t="str"/>
       <x:c r="P50" s="17" t="str"/>
+      <x:c r="Q50" t="str">
+        <x:v>内容进入前台并连续可见约 1 秒时记录一次；快速划过、预加载和同一页面实例同一内容重复出现不记录。参数用于说明内容模块、内容标识、位置及 ready/empty 状态。</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -2748,6 +2892,9 @@
       <x:c r="P51" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q51" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
@@ -2798,6 +2945,9 @@
       <x:c r="P52" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q52" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="24" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
@@ -2847,6 +2997,9 @@
       </x:c>
       <x:c r="P53" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q53" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="24" hidden="0" customHeight="1">
@@ -2884,6 +3037,9 @@
       <x:c r="N54" s="17" t="str"/>
       <x:c r="O54" s="17" t="str"/>
       <x:c r="P54" s="17" t="str"/>
+      <x:c r="Q54" t="str">
+        <x:v>提交请求收到明确接口终态时记录；点击按钮、校验通过或成功页加载都不能替代接口结果。selling_method、件数/品类/品牌/照片数量和日期/Referral 是否填写用于解释提交构成，result_state 用于区分成功、失败或取消。</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="24" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
@@ -2920,6 +3076,9 @@
       <x:c r="N55" s="17" t="str"/>
       <x:c r="O55" s="17" t="str"/>
       <x:c r="P55" s="17" t="str"/>
+      <x:c r="Q55" t="str">
+        <x:v>提交请求收到明确接口终态时记录；点击按钮、校验通过或成功页加载都不能替代接口结果。selling_method、件数/品类/品牌/照片数量和日期/Referral 是否填写用于解释提交构成，result_state 用于区分成功、失败或取消。</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -2969,6 +3128,9 @@
       </x:c>
       <x:c r="P56" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q56" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
@@ -3006,6 +3168,9 @@
       <x:c r="N57" s="17" t="str"/>
       <x:c r="O57" s="17" t="str"/>
       <x:c r="P57" s="17" t="str"/>
+      <x:c r="Q57" t="str">
+        <x:v>后台权威预约记录创建成功时记录一次；按 request_id 去重。它表示后台事实，不等同于前台点击提交，业务上用于统计真实创建量和与前台提交结果分开对账。</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
@@ -3042,6 +3207,9 @@
       <x:c r="N58" s="17" t="str"/>
       <x:c r="O58" s="17" t="str"/>
       <x:c r="P58" s="17" t="str"/>
+      <x:c r="Q58" t="str">
+        <x:v>页面实例真正到达并可见时记录；预加载、后台预取和同一页面实例重复渲染不算新的到达。参数用于标识页面（page_id）、页面实例（page_instance_id）和后续来源/设备分析。</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
@@ -3092,6 +3260,9 @@
       <x:c r="P59" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q59" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
@@ -3142,6 +3313,9 @@
       <x:c r="P60" s="17" t="str">
         <x:v>fill</x:v>
       </x:c>
+      <x:c r="Q60" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
@@ -3192,6 +3366,9 @@
       <x:c r="P61" s="17" t="str">
         <x:v>validation</x:v>
       </x:c>
+      <x:c r="Q61" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
@@ -3242,6 +3419,9 @@
       <x:c r="P62" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q62" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="12" t="str">
@@ -3292,6 +3472,9 @@
       <x:c r="P63" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q63" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="12" t="str">
@@ -3342,6 +3525,9 @@
       <x:c r="P64" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q64" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
@@ -3392,6 +3578,9 @@
       <x:c r="P65" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q65" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="12" t="str">
@@ -3442,6 +3631,9 @@
       <x:c r="P66" s="17" t="str">
         <x:v>default</x:v>
       </x:c>
+      <x:c r="Q66" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="12" t="str">
@@ -3491,6 +3683,9 @@
       </x:c>
       <x:c r="P67" s="17" t="str">
         <x:v>default</x:v>
+      </x:c>
+      <x:c r="Q67" t="str">
+        <x:v>用户完成该控件的稳定业务操作时记录；焦点移动、逐字输入和无业务结果的点击不记录。interaction_name/action/element_id 说明做了什么，page_id/module_id 说明发生在哪里，其他字段补充该操作的业务选择或结果。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5192,6 +5387,9 @@
       <x:c r="F3" s="21" t="str">
         <x:v>明确不上报</x:v>
       </x:c>
+      <x:c r="G3" t="str">
+        <x:v>业务解释（触发时机 / 参数意义）</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -5212,6 +5410,9 @@
       <x:c r="F4" s="13" t="str">
         <x:v>身份ID、完整ZIP；Session仍为全站</x:v>
       </x:c>
+      <x:c r="G4" t="str">
+        <x:v>C1 页面真实到达时上报，用来统计 Sell 页面流量；page_id/page_type 说明页面，business_domain=c1 用于从全站 GA4 中筛出 C1，locale/market/device_type/entry_source 用于按语言、市场、设备和入口比较。</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -5232,6 +5433,9 @@
       <x:c r="F5" s="13" t="str">
         <x:v>flow_id、入口event_id</x:v>
       </x:c>
+      <x:c r="G5" t="str">
+        <x:v>预约表单第一次真正展示时上报，表示用户进入卖货流程；entry_source 说明入口，prefilled_zip_present 和 preselected_method 说明流程是否带入已有信息，便于解释预约开始来源和预填状态。</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -5252,6 +5456,9 @@
       <x:c r="F6" s="13" t="str">
         <x:v>field原文、业务主键</x:v>
       </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Step 1–4 实际展示时上报，用来定位预约漏斗在哪一步流失；step_id 表示步骤，flow_scope/business_domain 用于限定 C1，device_type/locale 用于切分端和语言。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -5272,6 +5479,9 @@
       <x:c r="F7" s="13" t="str">
         <x:v>完整ZIP、coverage_check_id</x:v>
       </x:c>
+      <x:c r="G7" t="str">
+        <x:v>ZIP 查询出现明确终态时上报，用来分析服务覆盖对预约的影响；query_context 说明查询场景，result_state 说明请求是否成功，coverage_status 只在成功查询时表示 covered/uncovered，其余字段说明可用方式和是否重试。</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -5292,6 +5502,9 @@
       <x:c r="F8" s="13" t="str">
         <x:v>Flow ID、默认自动选择</x:v>
       </x:c>
+      <x:c r="G8" t="str">
+        <x:v>用户主动选择售卖方式时上报，用来比较 In-Home、Visit Looply、Ship To Us 的偏好；selling_method 是所选方式，selection_origin=user 排除系统默认推荐，step_id 说明发生在哪一步。</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
@@ -5311,6 +5524,9 @@
       </x:c>
       <x:c r="F9" s="15" t="str">
         <x:v>业务主键、联系方式（均不上传）</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>前台提交接口明确成功时上报并作为 GA4 关键事件；selling_method、piece_count_bucket、category_count、brand_count、photo_count 描述提交内容规模，coverage_status、preferred_date_present、referral_present 描述关键条件是否满足，result_state 固定为 success。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>